<commit_message>
feat(accel): add Price_Mismatch_Summary dynamic formula sheet and final page SKU/price mismatch validation
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/Accel_mode26-10-2026.xlsx
+++ b/projects/auto_page/autopageMKII/tables/Accel_mode26-10-2026.xlsx
@@ -488,7 +488,7 @@
   <dimension ref="A1:AY66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" style="4" min="1" max="1"/>
+    <col width="24" customWidth="1" style="4" min="1" max="1"/>
     <col width="12" customWidth="1" style="4" min="2" max="2"/>
     <col width="16" customWidth="1" style="4" min="3" max="3"/>
     <col width="17" customWidth="1" style="4" min="4" max="4"/>
@@ -4854,7 +4854,7 @@
   <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" style="4" min="1" max="1"/>
+    <col width="22" customWidth="1" style="4" min="1" max="1"/>
     <col width="20" customWidth="1" style="4" min="2" max="2"/>
     <col width="24" customWidth="1" style="4" min="3" max="3"/>
     <col width="24" customWidth="1" style="4" min="4" max="4"/>
@@ -4912,7 +4912,7 @@
         </is>
       </c>
     </row>
-    <row r="2" s="4">
+    <row r="2" hidden="1" s="4">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:35:11</t>
@@ -4951,7 +4951,7 @@
       <c r="H2" s="3" t="inlineStr"/>
       <c r="I2" s="3" t="inlineStr"/>
     </row>
-    <row r="3" s="4">
+    <row r="3" hidden="1" s="4">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:36:29</t>
@@ -4990,7 +4990,7 @@
       <c r="H3" s="3" t="inlineStr"/>
       <c r="I3" s="3" t="inlineStr"/>
     </row>
-    <row r="4" s="4">
+    <row r="4" hidden="1" s="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:37:50</t>
@@ -5029,7 +5029,7 @@
       <c r="H4" s="3" t="inlineStr"/>
       <c r="I4" s="3" t="inlineStr"/>
     </row>
-    <row r="5" s="4">
+    <row r="5" hidden="1" s="4">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:39:06</t>
@@ -5068,7 +5068,7 @@
       <c r="H5" s="3" t="inlineStr"/>
       <c r="I5" s="3" t="inlineStr"/>
     </row>
-    <row r="6" s="4">
+    <row r="6" hidden="1" s="4">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:40:06</t>
@@ -5107,7 +5107,7 @@
       <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr"/>
     </row>
-    <row r="7" s="4">
+    <row r="7" hidden="1" s="4">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:41:24</t>
@@ -5146,7 +5146,7 @@
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr"/>
     </row>
-    <row r="8" s="4">
+    <row r="8" hidden="1" s="4">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:42:33</t>
@@ -5185,7 +5185,7 @@
       <c r="H8" s="3" t="inlineStr"/>
       <c r="I8" s="3" t="inlineStr"/>
     </row>
-    <row r="9" s="4">
+    <row r="9" hidden="1" s="4">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:43:37</t>
@@ -5224,7 +5224,7 @@
       <c r="H9" s="3" t="inlineStr"/>
       <c r="I9" s="3" t="inlineStr"/>
     </row>
-    <row r="10" s="4">
+    <row r="10" hidden="1" s="4">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:44:33</t>
@@ -5263,7 +5263,7 @@
       <c r="H10" s="3" t="inlineStr"/>
       <c r="I10" s="3" t="inlineStr"/>
     </row>
-    <row r="11" s="4">
+    <row r="11" hidden="1" s="4">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:45:29</t>
@@ -5302,7 +5302,7 @@
       <c r="H11" s="3" t="inlineStr"/>
       <c r="I11" s="3" t="inlineStr"/>
     </row>
-    <row r="12" s="4">
+    <row r="12" hidden="1" s="4">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:46:26</t>
@@ -5341,7 +5341,7 @@
       <c r="H12" s="3" t="inlineStr"/>
       <c r="I12" s="3" t="inlineStr"/>
     </row>
-    <row r="13" s="4">
+    <row r="13" hidden="1" s="4">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:47:22</t>
@@ -5380,7 +5380,7 @@
       <c r="H13" s="3" t="inlineStr"/>
       <c r="I13" s="3" t="inlineStr"/>
     </row>
-    <row r="14" s="4">
+    <row r="14" hidden="1" s="4">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:48:16</t>
@@ -5419,7 +5419,7 @@
       <c r="H14" s="3" t="inlineStr"/>
       <c r="I14" s="3" t="inlineStr"/>
     </row>
-    <row r="15" s="4">
+    <row r="15" hidden="1" s="4">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:49:19</t>
@@ -5458,7 +5458,7 @@
       <c r="H15" s="3" t="inlineStr"/>
       <c r="I15" s="3" t="inlineStr"/>
     </row>
-    <row r="16" s="4">
+    <row r="16" hidden="1" s="4">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:50:20</t>
@@ -5497,7 +5497,7 @@
       <c r="H16" s="3" t="inlineStr"/>
       <c r="I16" s="3" t="inlineStr"/>
     </row>
-    <row r="17" s="4">
+    <row r="17" hidden="1" s="4">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:51:13</t>
@@ -5536,7 +5536,7 @@
       <c r="H17" s="3" t="inlineStr"/>
       <c r="I17" s="3" t="inlineStr"/>
     </row>
-    <row r="18" s="4">
+    <row r="18" hidden="1" s="4">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:52:14</t>
@@ -5575,7 +5575,7 @@
       <c r="H18" s="3" t="inlineStr"/>
       <c r="I18" s="3" t="inlineStr"/>
     </row>
-    <row r="19" s="4">
+    <row r="19" hidden="1" s="4">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:53:07</t>
@@ -5614,7 +5614,7 @@
       <c r="H19" s="3" t="inlineStr"/>
       <c r="I19" s="3" t="inlineStr"/>
     </row>
-    <row r="20" s="4">
+    <row r="20" hidden="1" s="4">
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:54:01</t>
@@ -5653,7 +5653,7 @@
       <c r="H20" s="3" t="inlineStr"/>
       <c r="I20" s="3" t="inlineStr"/>
     </row>
-    <row r="21" s="4">
+    <row r="21" hidden="1" s="4">
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:54:58</t>
@@ -5692,7 +5692,7 @@
       <c r="H21" s="3" t="inlineStr"/>
       <c r="I21" s="3" t="inlineStr"/>
     </row>
-    <row r="22" s="4">
+    <row r="22" hidden="1" s="4">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:55:54</t>
@@ -5731,7 +5731,7 @@
       <c r="H22" s="3" t="inlineStr"/>
       <c r="I22" s="3" t="inlineStr"/>
     </row>
-    <row r="23" s="4">
+    <row r="23" hidden="1" s="4">
       <c r="A23" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:56:52</t>
@@ -5770,7 +5770,7 @@
       <c r="H23" s="3" t="inlineStr"/>
       <c r="I23" s="3" t="inlineStr"/>
     </row>
-    <row r="24" s="4">
+    <row r="24" hidden="1" s="4">
       <c r="A24" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:57:46</t>
@@ -5809,7 +5809,7 @@
       <c r="H24" s="3" t="inlineStr"/>
       <c r="I24" s="3" t="inlineStr"/>
     </row>
-    <row r="25" s="4">
+    <row r="25" hidden="1" s="4">
       <c r="A25" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:58:39</t>
@@ -5848,7 +5848,7 @@
       <c r="H25" s="3" t="inlineStr"/>
       <c r="I25" s="3" t="inlineStr"/>
     </row>
-    <row r="26" s="4">
+    <row r="26" hidden="1" s="4">
       <c r="A26" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 15:59:36</t>
@@ -5887,7 +5887,7 @@
       <c r="H26" s="3" t="inlineStr"/>
       <c r="I26" s="3" t="inlineStr"/>
     </row>
-    <row r="27" s="4">
+    <row r="27" hidden="1" s="4">
       <c r="A27" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 16:00:33</t>
@@ -5926,7 +5926,7 @@
       <c r="H27" s="3" t="inlineStr"/>
       <c r="I27" s="3" t="inlineStr"/>
     </row>
-    <row r="28" s="4">
+    <row r="28" hidden="1" s="4">
       <c r="A28" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 16:01:31</t>
@@ -5965,7 +5965,7 @@
       <c r="H28" s="3" t="inlineStr"/>
       <c r="I28" s="3" t="inlineStr"/>
     </row>
-    <row r="29" s="4">
+    <row r="29" hidden="1" s="4">
       <c r="A29" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 16:02:27</t>
@@ -6004,7 +6004,7 @@
       <c r="H29" s="3" t="inlineStr"/>
       <c r="I29" s="3" t="inlineStr"/>
     </row>
-    <row r="30" s="4">
+    <row r="30" hidden="1" s="4">
       <c r="A30" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 16:03:22</t>
@@ -6043,7 +6043,7 @@
       <c r="H30" s="3" t="inlineStr"/>
       <c r="I30" s="3" t="inlineStr"/>
     </row>
-    <row r="31" s="4">
+    <row r="31" hidden="1" s="4">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 16:04:19</t>
@@ -6082,7 +6082,7 @@
       <c r="H31" s="3" t="inlineStr"/>
       <c r="I31" s="3" t="inlineStr"/>
     </row>
-    <row r="32" s="4">
+    <row r="32" hidden="1" s="4">
       <c r="A32" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 16:05:23</t>
@@ -6121,7 +6121,7 @@
       <c r="H32" s="3" t="inlineStr"/>
       <c r="I32" s="3" t="inlineStr"/>
     </row>
-    <row r="33" s="4">
+    <row r="33" hidden="1" s="4">
       <c r="A33" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 16:06:17</t>
@@ -6160,7 +6160,7 @@
       <c r="H33" s="3" t="inlineStr"/>
       <c r="I33" s="3" t="inlineStr"/>
     </row>
-    <row r="34" s="4">
+    <row r="34" hidden="1" s="4">
       <c r="A34" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 16:07:13</t>
@@ -6199,7 +6199,7 @@
       <c r="H34" s="3" t="inlineStr"/>
       <c r="I34" s="3" t="inlineStr"/>
     </row>
-    <row r="35" s="4">
+    <row r="35" hidden="1" s="4">
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 16:08:09</t>
@@ -6253,7 +6253,7 @@
   <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" style="4" min="1" max="1"/>
+    <col width="22" customWidth="1" style="4" min="1" max="1"/>
     <col width="24" customWidth="1" style="4" min="2" max="2"/>
     <col width="15" customWidth="1" style="4" min="3" max="3"/>
   </cols>

</xml_diff>

<commit_message>
feat(pricing): add order date filtering, base price pre-discount recovery, and auto oc/dc adjustment
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/Accel_mode26-10-2026.xlsx
+++ b/projects/auto_page/autopageMKII/tables/Accel_mode26-10-2026.xlsx
@@ -488,7 +488,7 @@
   <dimension ref="A1:AY66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="4" min="1" max="1"/>
+    <col width="32" customWidth="1" style="4" min="1" max="1"/>
     <col width="12" customWidth="1" style="4" min="2" max="2"/>
     <col width="16" customWidth="1" style="4" min="3" max="3"/>
     <col width="17" customWidth="1" style="4" min="4" max="4"/>
@@ -4854,7 +4854,7 @@
   <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" style="4" min="1" max="1"/>
+    <col width="32" customWidth="1" style="4" min="1" max="1"/>
     <col width="20" customWidth="1" style="4" min="2" max="2"/>
     <col width="24" customWidth="1" style="4" min="3" max="3"/>
     <col width="24" customWidth="1" style="4" min="4" max="4"/>
@@ -6253,7 +6253,7 @@
   <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" style="4" min="1" max="1"/>
+    <col width="32" customWidth="1" style="4" min="1" max="1"/>
     <col width="24" customWidth="1" style="4" min="2" max="2"/>
     <col width="15" customWidth="1" style="4" min="3" max="3"/>
   </cols>

</xml_diff>